<commit_message>
Updated to fall date and updated format of Template card to add data validation
</commit_message>
<xml_diff>
--- a/Template Comment Card Sheet.xlsx
+++ b/Template Comment Card Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30317"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hunsber3\Development\UofT-Report-Cards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2D3F7D0-8035-4CA6-A8C8-E5A693C69D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CA94004-2EA3-415A-9C77-F331E29408AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="12735" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="12735" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Swimmers" sheetId="1" r:id="rId1"/>
@@ -32,15 +32,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Name:</t>
   </si>
@@ -109,6 +106,12 @@
   </si>
   <si>
     <t>Swim for Life 10</t>
+  </si>
+  <si>
+    <t>Swim for Life 9 or Intro to Competitive Swimming</t>
+  </si>
+  <si>
+    <t>Bronze Star/Bronze Medallion</t>
   </si>
 </sst>
 </file>
@@ -118,7 +121,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -127,15 +130,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -143,16 +158,164 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -467,47 +630,438 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F49"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38" style="1" customWidth="1"/>
+    <col min="4" max="4" width="20.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="7"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="8"/>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="7"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="8"/>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="7"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="8"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="7"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="8"/>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="7"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="8"/>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="7"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="8"/>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="7"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="8"/>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="7"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="8"/>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="7"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="12"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="8"/>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="7"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="8"/>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="7"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="8"/>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="7"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="8"/>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="7"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="8"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="7"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="8"/>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="7"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="8"/>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="7"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="8"/>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="7"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="8"/>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="7"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="8"/>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="7"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="8"/>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="7"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="8"/>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="7"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="8"/>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="7"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="8"/>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="7"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="8"/>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="7"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="8"/>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="7"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="8"/>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" s="7"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="8"/>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="7"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="8"/>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" s="7"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="8"/>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="7"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="8"/>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="7"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="8"/>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="7"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="8"/>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="7"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" s="7"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="8"/>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="7"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="12"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="8"/>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="7"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="8"/>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" s="7"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="8"/>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="7"/>
+      <c r="B38" s="3"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="8"/>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="7"/>
+      <c r="B39" s="3"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="8"/>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="7"/>
+      <c r="B40" s="3"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="8"/>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="7"/>
+      <c r="B41" s="3"/>
+      <c r="C41" s="12"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="8"/>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="7"/>
+      <c r="B42" s="3"/>
+      <c r="C42" s="12"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="8"/>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="7"/>
+      <c r="B43" s="3"/>
+      <c r="C43" s="12"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="8"/>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" s="7"/>
+      <c r="B44" s="3"/>
+      <c r="C44" s="12"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="8"/>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="7"/>
+      <c r="B45" s="3"/>
+      <c r="C45" s="12"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="8"/>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="7"/>
+      <c r="B46" s="3"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="8"/>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" s="7"/>
+      <c r="B47" s="3"/>
+      <c r="C47" s="12"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="8"/>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" s="7"/>
+      <c r="B48" s="3"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="8"/>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="9"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8326298D-966F-4672-8F4E-6071AEF56D2D}">
           <x14:formula1>
             <xm:f>Reference!$B$2:$B$17</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B40</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{24971310-9D18-43C2-9420-A4DFD850338A}">
+          <x14:formula1>
+            <xm:f>Reference!$B$2:$B$19</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2:D49</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -517,202 +1071,103 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{845B324E-861F-42A9-AC46-555DA09A1FE6}">
-  <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:B19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="2:2">
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="2" spans="2:2">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="3" t="s">
+    </row>
+    <row r="3" spans="2:2">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="3" t="s">
+    </row>
+    <row r="4" spans="2:2">
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="3" t="s">
+    </row>
+    <row r="5" spans="2:2">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="3" t="s">
+    </row>
+    <row r="6" spans="2:2">
+      <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="3" t="s">
+    </row>
+    <row r="7" spans="2:2">
+      <c r="B7" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="3" t="s">
+    </row>
+    <row r="8" spans="2:2">
+      <c r="B8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3" t="s">
+    </row>
+    <row r="9" spans="2:2">
+      <c r="B9" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="3" t="s">
+    </row>
+    <row r="10" spans="2:2">
+      <c r="B10" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="3" t="s">
+    </row>
+    <row r="11" spans="2:2">
+      <c r="B11" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="3" t="s">
+    </row>
+    <row r="12" spans="2:2">
+      <c r="B12" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="3" t="s">
+    </row>
+    <row r="13" spans="2:2">
+      <c r="B13" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="3" t="s">
+    </row>
+    <row r="14" spans="2:2">
+      <c r="B14" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="3" t="s">
+    </row>
+    <row r="15" spans="2:2">
+      <c r="B15" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="3" t="s">
+    </row>
+    <row r="16" spans="2:2">
+      <c r="B16" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="3" t="s">
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+    </row>
+    <row r="18" spans="2:2">
+      <c r="B18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19" t="s">
+        <v>24</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -720,21 +1175,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="56e547ad-939e-48f8-beb4-e3c72ca314ea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9a31eef5-a1f4-43e4-ae7b-bfb699e14659" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100435CF8FC1F9D314D954D997B962F9723" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f416500480350d3fd550bc6e09077061">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="56e547ad-939e-48f8-beb4-e3c72ca314ea" xmlns:ns3="9a31eef5-a1f4-43e4-ae7b-bfb699e14659" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2b295d93146c64d94a22fdabffd16a72" ns2:_="" ns3:_="">
-    <xsd:import namespace="56e547ad-939e-48f8-beb4-e3c72ca314ea"/>
-    <xsd:import namespace="9a31eef5-a1f4-43e4-ae7b-bfb699e14659"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BEAE441166E2E947A16064CC9D141789" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4f1dc8434ba1b11f414d893867e53a89">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0b95d19c-9c53-4ddc-b525-7fb311e47dec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4461b1d7dd8ac0764a35a570578d2c4e" ns2:_="">
+    <xsd:import namespace="0b95d19c-9c53-4ddc-b525-7fb311e47dec"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -744,16 +1196,11 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -761,7 +1208,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="56e547ad-939e-48f8-beb4-e3c72ca314ea" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="0b95d19c-9c53-4ddc-b525-7fb311e47dec" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -779,69 +1226,30 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="12" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="14" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="17" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="fe164b29-4069-4387-b6aa-f01f2a1f4743" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="19" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaLengthInSeconds" ma:index="15" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
       <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
+        <xsd:restriction base="dms:Unknown"/>
       </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="20" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="21" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9a31eef5-a1f4-43e4-ae7b-bfb699e14659" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="18" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{d83a7c06-7d99-49a1-9d1a-e7ea7e5444d4}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="9a31eef5-a1f4-43e4-ae7b-bfb699e14659">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -944,48 +1352,19 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F06C923D-4E57-4D2D-B29F-1518299C6FAE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="56e547ad-939e-48f8-beb4-e3c72ca314ea"/>
-    <ds:schemaRef ds:uri="9a31eef5-a1f4-43e4-ae7b-bfb699e14659"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D74BEB-6D96-4C6A-84FA-A4054BA23F01}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{44C6EEEA-0051-440B-8A67-12033724E6D3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="56e547ad-939e-48f8-beb4-e3c72ca314ea"/>
-    <ds:schemaRef ds:uri="9a31eef5-a1f4-43e4-ae7b-bfb699e14659"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37D2D62C-5747-4A72-9D0F-B10ED49D7439}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D74BEB-6D96-4C6A-84FA-A4054BA23F01}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F06C923D-4E57-4D2D-B29F-1518299C6FAE}"/>
 </file>
</xml_diff>